<commit_message>
removed unused files from Vivado project
</commit_message>
<xml_diff>
--- a/project/graphic_designing/encoded_letters.xlsx
+++ b/project/graphic_designing/encoded_letters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joelk\Documents\ee_files\EE2026\project\graphic_designing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1392200-F42B-465C-BEB9-A0A0A4C09B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A50F4E-A826-4F66-A277-96125A9AC39E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28665" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="1" xr2:uid="{3F09DA75-48F6-4CED-A1E4-6F4F2B560964}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F09DA75-48F6-4CED-A1E4-6F4F2B560964}"/>
   </bookViews>
   <sheets>
     <sheet name="Letter Encoding" sheetId="1" r:id="rId1"/>
@@ -7408,5 +7408,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>